<commit_message>
feat: Made file names consistent. Improved printing of discrepancies.
</commit_message>
<xml_diff>
--- a/examples2/2_leahQualifiersTemplate.xlsx
+++ b/examples2/2_leahQualifiersTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryan\Desktop\ESC\HouseChamps\examples2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E143E7E3-9FBD-4A99-A181-AD299C3DD252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14637EC8-F66A-425B-9CA9-69355593341C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{E1B62AB6-8038-40A9-A8B0-597DE2503C4A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3986" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4656" uniqueCount="831">
   <si>
     <t>Acton Spring House Champs Heats</t>
   </si>
@@ -2388,13 +2388,154 @@
   </si>
   <si>
     <t>Event  41   Girls 9 &amp; Under 100 SC Meter IM</t>
+  </si>
+  <si>
+    <t>Event  51   Girls 200 SC Meter IM</t>
+  </si>
+  <si>
+    <t>Heat   1 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   2 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   3 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   4 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   5 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   6 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   7 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>4:43.19</t>
+  </si>
+  <si>
+    <t>4:44.97</t>
+  </si>
+  <si>
+    <t>Heat   8 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>4:16.06</t>
+  </si>
+  <si>
+    <t>3:58.91</t>
+  </si>
+  <si>
+    <t>3:49.97</t>
+  </si>
+  <si>
+    <t>3:48.56</t>
+  </si>
+  <si>
+    <t>3:56.97</t>
+  </si>
+  <si>
+    <t>4:10.63</t>
+  </si>
+  <si>
+    <t>4:16.44</t>
+  </si>
+  <si>
+    <t>Heat   9 of 9   Timed Finals</t>
+  </si>
+  <si>
+    <t>3:40.37</t>
+  </si>
+  <si>
+    <t>3:33.38</t>
+  </si>
+  <si>
+    <t>2:58.22</t>
+  </si>
+  <si>
+    <t>2:43.93</t>
+  </si>
+  <si>
+    <t>2:57.60</t>
+  </si>
+  <si>
+    <t>3:31.72</t>
+  </si>
+  <si>
+    <t>3:40.32</t>
+  </si>
+  <si>
+    <t>3:40.56</t>
+  </si>
+  <si>
+    <t>Event  52   Open/Boys 200 SC Meter IM</t>
+  </si>
+  <si>
+    <t>Heat   1 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   2 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   3 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   4 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   5 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>Heat   6 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>3:49.35</t>
+  </si>
+  <si>
+    <t>3:33.81</t>
+  </si>
+  <si>
+    <t>3:43.44</t>
+  </si>
+  <si>
+    <t>4:09.94</t>
+  </si>
+  <si>
+    <t>Heat   7 of 7   Timed Finals</t>
+  </si>
+  <si>
+    <t>3:14.45</t>
+  </si>
+  <si>
+    <t>3:12.24</t>
+  </si>
+  <si>
+    <t>3:02.48</t>
+  </si>
+  <si>
+    <t>2:55.81</t>
+  </si>
+  <si>
+    <t>2:56.66</t>
+  </si>
+  <si>
+    <t>3:05.03</t>
+  </si>
+  <si>
+    <t>3:12.63</t>
+  </si>
+  <si>
+    <t>3:18.38</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2422,6 +2563,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="ARIAL"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2431,7 +2603,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -2454,6 +2626,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2462,7 +2677,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1">
       <alignment vertical="top"/>
@@ -2487,6 +2702,66 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2825,7 +3100,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FD61760-8120-4FFC-BC04-B52E600A0D89}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F969"/>
+  <dimension ref="A1:F1128"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="61.19921875" bestFit="1" customWidth="1"/>
@@ -18241,6 +18516,2586 @@
       </c>
       <c r="F969"/>
     </row>
+    <row r="971" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A971" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="B971" s="3"/>
+      <c r="C971" s="3"/>
+      <c r="D971" s="4"/>
+      <c r="E971" s="3"/>
+      <c r="F971" s="3"/>
+    </row>
+    <row r="972" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A972" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B972" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C972" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D972" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E972" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F972" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="973" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A973" s="5" t="s">
+        <v>785</v>
+      </c>
+      <c r="B973" s="5"/>
+      <c r="C973" s="5"/>
+      <c r="D973" s="6"/>
+      <c r="E973" s="5"/>
+      <c r="F973" s="5"/>
+    </row>
+    <row r="974" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A974" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B974" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C974" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D974" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E974" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F974" s="5"/>
+    </row>
+    <row r="975" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A975" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B975" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C975" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D975" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E975" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F975" s="5"/>
+    </row>
+    <row r="976" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A976" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B976" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C976" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D976" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E976" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F976" s="9"/>
+    </row>
+    <row r="977" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A977" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B977" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C977" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D977" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E977" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F977" s="5"/>
+    </row>
+    <row r="978" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A978" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B978" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C978" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D978" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E978" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F978" s="5"/>
+    </row>
+    <row r="979" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A979" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B979" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C979" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D979" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E979" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F979" s="5"/>
+    </row>
+    <row r="980" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A980" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B980" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C980" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D980" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E980" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F980" s="5"/>
+    </row>
+    <row r="981" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A981" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B981" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C981" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D981" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E981" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F981" s="5"/>
+    </row>
+    <row r="982" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A982" s="5" t="s">
+        <v>786</v>
+      </c>
+      <c r="B982" s="5"/>
+      <c r="C982" s="5"/>
+      <c r="D982" s="6"/>
+      <c r="E982" s="5"/>
+      <c r="F982" s="5"/>
+    </row>
+    <row r="983" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A983" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B983" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C983" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D983" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E983" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F983" s="5"/>
+    </row>
+    <row r="984" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A984" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B984" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C984" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D984" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E984" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F984" s="5"/>
+    </row>
+    <row r="985" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A985" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B985" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C985" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D985" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E985" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F985" s="5"/>
+    </row>
+    <row r="986" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A986" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B986" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C986" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D986" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E986" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F986" s="5"/>
+    </row>
+    <row r="987" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A987" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B987" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C987" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D987" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E987" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F987" s="5"/>
+    </row>
+    <row r="988" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A988" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B988" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C988" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D988" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E988" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F988" s="5"/>
+    </row>
+    <row r="989" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A989" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B989" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C989" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D989" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E989" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F989" s="5"/>
+    </row>
+    <row r="990" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A990" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B990" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C990" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D990" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E990" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F990" s="5"/>
+    </row>
+    <row r="991" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A991" s="5" t="s">
+        <v>787</v>
+      </c>
+      <c r="B991" s="5"/>
+      <c r="C991" s="5"/>
+      <c r="D991" s="6"/>
+      <c r="E991" s="5"/>
+      <c r="F991" s="5"/>
+    </row>
+    <row r="992" spans="1:6" ht="21.4" x14ac:dyDescent="0.8">
+      <c r="A992" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B992" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C992" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D992" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E992" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F992" s="10"/>
+    </row>
+    <row r="993" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A993" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B993" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C993" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D993" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E993" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F993" s="5"/>
+    </row>
+    <row r="994" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A994" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B994" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C994" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D994" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E994" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F994" s="5"/>
+    </row>
+    <row r="995" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A995" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B995" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C995" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D995" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E995" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F995" s="5"/>
+    </row>
+    <row r="996" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A996" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B996" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C996" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D996" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E996" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F996" s="5"/>
+    </row>
+    <row r="997" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A997" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B997" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C997" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D997" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E997" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F997" s="5"/>
+    </row>
+    <row r="998" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A998" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B998" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C998" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D998" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E998" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F998" s="5"/>
+    </row>
+    <row r="999" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A999" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B999" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C999" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D999" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E999" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F999" s="5"/>
+    </row>
+    <row r="1000" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1000" s="5" t="s">
+        <v>788</v>
+      </c>
+      <c r="B1000" s="5"/>
+      <c r="C1000" s="5"/>
+      <c r="D1000" s="6"/>
+      <c r="E1000" s="5"/>
+      <c r="F1000" s="5"/>
+    </row>
+    <row r="1001" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1001" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1001" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1001" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1001" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1001" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1001" s="11"/>
+    </row>
+    <row r="1002" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1002" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1002" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1002" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1002" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1002" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1002" s="5"/>
+    </row>
+    <row r="1003" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1003" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1003" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1003" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1003" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1003" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1003" s="5"/>
+    </row>
+    <row r="1004" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1004" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1004" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1004" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1004" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1004" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1004" s="5"/>
+    </row>
+    <row r="1005" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1005" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1005" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1005" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1005" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1005" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1005" s="11"/>
+    </row>
+    <row r="1006" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1006" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1006" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1006" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1006" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1006" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1006" s="5"/>
+    </row>
+    <row r="1007" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1007" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1007" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1007" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1007" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1007" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1007" s="5"/>
+    </row>
+    <row r="1008" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1008" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1008" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1008" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1008" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1008" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1008" s="11"/>
+    </row>
+    <row r="1009" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1009" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="B1009" s="5"/>
+      <c r="C1009" s="5"/>
+      <c r="D1009" s="6"/>
+      <c r="E1009" s="5"/>
+      <c r="F1009" s="5"/>
+    </row>
+    <row r="1010" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1010" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1010" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1010" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1010" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1010" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1010" s="5"/>
+    </row>
+    <row r="1011" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1011" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1011" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1011" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1011" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1011" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1011" s="5"/>
+    </row>
+    <row r="1012" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1012" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1012" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1012" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1012" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1012" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1012" s="5"/>
+    </row>
+    <row r="1013" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1013" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1013" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C1013" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1013" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1013" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1013" s="5"/>
+    </row>
+    <row r="1014" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1014" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1014" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1014" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1014" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1014" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1014" s="5"/>
+    </row>
+    <row r="1015" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1015" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1015" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1015" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1015" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1015" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1015" s="5"/>
+    </row>
+    <row r="1016" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1016" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1016" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1016" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1016" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1016" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1016" s="5"/>
+    </row>
+    <row r="1017" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1017" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1017" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1017" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1017" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1017" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1017" s="5"/>
+    </row>
+    <row r="1018" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1018" s="5" t="s">
+        <v>790</v>
+      </c>
+      <c r="B1018" s="5"/>
+      <c r="C1018" s="5"/>
+      <c r="D1018" s="6"/>
+      <c r="E1018" s="5"/>
+      <c r="F1018" s="5"/>
+    </row>
+    <row r="1019" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1019" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1019" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1019" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1019" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1019" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1019" s="11"/>
+    </row>
+    <row r="1020" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1020" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1020" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1020" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1020" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1020" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1020" s="5"/>
+    </row>
+    <row r="1021" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1021" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1021" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1021" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1021" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1021" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1021" s="5"/>
+    </row>
+    <row r="1022" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1022" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1022" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1022" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1022" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1022" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1022" s="5"/>
+    </row>
+    <row r="1023" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1023" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1023" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1023" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1023" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1023" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1023" s="5"/>
+    </row>
+    <row r="1024" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1024" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1024" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1024" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1024" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1024" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1024" s="5"/>
+    </row>
+    <row r="1025" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1025" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1025" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1025" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1025" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1025" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1025" s="5"/>
+    </row>
+    <row r="1026" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1026" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1026" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1026" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1026" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1026" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1026" s="5"/>
+    </row>
+    <row r="1027" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1027" s="5" t="s">
+        <v>791</v>
+      </c>
+      <c r="B1027" s="5"/>
+      <c r="C1027" s="5"/>
+      <c r="D1027" s="6"/>
+      <c r="E1027" s="5"/>
+      <c r="F1027" s="5"/>
+    </row>
+    <row r="1028" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1028" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1028" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1028" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1028" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1028" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1028" s="5"/>
+    </row>
+    <row r="1029" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1029" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1029" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C1029" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1029" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1029" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1029" s="5"/>
+    </row>
+    <row r="1030" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1030" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1030" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1030" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1030" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1030" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1030" s="5"/>
+    </row>
+    <row r="1031" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1031" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1031" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1031" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1031" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1031" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="F1031" s="5"/>
+    </row>
+    <row r="1032" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1032" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1032" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1032" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1032" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1032" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="F1032" s="9"/>
+    </row>
+    <row r="1033" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1033" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1033" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C1033" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1033" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1033" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1033" s="5"/>
+    </row>
+    <row r="1034" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1034" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1034" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1034" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1034" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1034" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1034" s="5"/>
+    </row>
+    <row r="1035" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1035" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1035" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1035" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1035" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1035" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1035" s="5"/>
+    </row>
+    <row r="1036" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1036" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="B1036" s="5"/>
+      <c r="C1036" s="5"/>
+      <c r="D1036" s="6"/>
+      <c r="E1036" s="5"/>
+      <c r="F1036" s="5"/>
+    </row>
+    <row r="1037" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1037" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1037" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1037" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1037" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1037" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="F1037" s="11"/>
+    </row>
+    <row r="1038" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1038" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1038" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1038" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1038" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1038" s="5" t="s">
+        <v>796</v>
+      </c>
+      <c r="F1038" s="5"/>
+    </row>
+    <row r="1039" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1039" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1039" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1039" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1039" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1039" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="F1039" s="11"/>
+    </row>
+    <row r="1040" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1040" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1040" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1040" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1040" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1040" s="5" t="s">
+        <v>798</v>
+      </c>
+      <c r="F1040" s="5"/>
+    </row>
+    <row r="1041" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1041" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1041" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1041" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1041" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1041" s="5" t="s">
+        <v>798</v>
+      </c>
+      <c r="F1041" s="5"/>
+    </row>
+    <row r="1042" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1042" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1042" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1042" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1042" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1042" s="5" t="s">
+        <v>799</v>
+      </c>
+      <c r="F1042" s="11"/>
+    </row>
+    <row r="1043" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1043" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1043" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1043" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1043" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1043" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="F1043" s="5"/>
+    </row>
+    <row r="1044" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1044" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1044" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1044" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1044" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1044" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="F1044" s="9"/>
+    </row>
+    <row r="1045" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1045" s="5" t="s">
+        <v>802</v>
+      </c>
+      <c r="B1045" s="5"/>
+      <c r="C1045" s="5"/>
+      <c r="D1045" s="6"/>
+      <c r="E1045" s="5"/>
+      <c r="F1045" s="5"/>
+    </row>
+    <row r="1046" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1046" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1046" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1046" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1046" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1046" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="F1046" s="5"/>
+    </row>
+    <row r="1047" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1047" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1047" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1047" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1047" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1047" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="F1047" s="5"/>
+    </row>
+    <row r="1048" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1048" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1048" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1048" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1048" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1048" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="F1048" s="5"/>
+    </row>
+    <row r="1049" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1049" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1049" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1049" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1049" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1049" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="F1049" s="11"/>
+    </row>
+    <row r="1050" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1050" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1050" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="C1050" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1050" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1050" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="F1050" s="11"/>
+    </row>
+    <row r="1051" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1051" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1051" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C1051" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1051" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1051" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="F1051" s="5"/>
+    </row>
+    <row r="1052" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1052" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1052" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C1052" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1052" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1052" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="F1052" s="5"/>
+    </row>
+    <row r="1053" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.8">
+      <c r="A1053" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1053" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1053" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1053" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1053" s="5" t="s">
+        <v>810</v>
+      </c>
+      <c r="F1053" s="12"/>
+    </row>
+    <row r="1054" spans="1:6" ht="21.4" x14ac:dyDescent="0.8">
+      <c r="A1054" s="25"/>
+      <c r="B1054" s="26"/>
+      <c r="C1054" s="26"/>
+      <c r="D1054" s="27"/>
+      <c r="E1054" s="26"/>
+      <c r="F1054" s="28"/>
+    </row>
+    <row r="1055" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1055" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="B1055" s="3"/>
+      <c r="C1055" s="3"/>
+      <c r="D1055" s="4"/>
+      <c r="E1055" s="3"/>
+      <c r="F1055" s="3"/>
+    </row>
+    <row r="1056" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1056" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1056" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1056" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1056" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1056" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1056" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1057" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="B1057" s="5"/>
+      <c r="C1057" s="5"/>
+      <c r="D1057" s="6"/>
+      <c r="E1057" s="5"/>
+      <c r="F1057" s="5"/>
+    </row>
+    <row r="1058" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1058" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1058" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1058" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1058" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1058" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1058" s="5"/>
+    </row>
+    <row r="1059" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1059" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1059" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1059" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1059" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1059" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1059" s="5"/>
+    </row>
+    <row r="1060" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1060" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1060" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1060" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1060" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1060" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1060" s="11"/>
+    </row>
+    <row r="1061" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1061" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1061" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1061" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1061" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1061" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1061" s="5"/>
+    </row>
+    <row r="1062" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1062" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1062" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1062" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1062" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1062" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1062" s="5"/>
+    </row>
+    <row r="1063" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1063" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1063" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1063" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1063" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1063" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1063" s="5"/>
+    </row>
+    <row r="1064" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1064" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1064" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1064" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1064" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1064" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1064" s="5"/>
+    </row>
+    <row r="1065" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1065" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1065" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1065" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1065" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1065" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1065" s="5"/>
+    </row>
+    <row r="1066" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1066" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="B1066" s="5"/>
+      <c r="C1066" s="5"/>
+      <c r="D1066" s="6"/>
+      <c r="E1066" s="5"/>
+      <c r="F1066" s="5"/>
+    </row>
+    <row r="1067" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1067" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1067" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1067" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1067" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1067" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1067" s="5"/>
+    </row>
+    <row r="1068" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1068" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1068" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1068" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1068" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1068" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1068" s="5"/>
+    </row>
+    <row r="1069" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1069" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1069" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1069" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1069" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1069" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1069" s="5"/>
+    </row>
+    <row r="1070" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1070" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1070" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1070" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1070" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1070" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1070" s="5"/>
+    </row>
+    <row r="1071" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1071" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1071" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1071" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1071" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1071" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1071" s="5"/>
+    </row>
+    <row r="1072" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1072" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1072" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1072" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1072" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1072" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1072" s="5"/>
+    </row>
+    <row r="1073" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1073" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1073" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1073" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1073" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1073" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1073" s="11"/>
+    </row>
+    <row r="1074" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1074" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1074" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1074" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1074" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1074" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1074" s="5"/>
+    </row>
+    <row r="1075" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1075" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="B1075" s="5"/>
+      <c r="C1075" s="5"/>
+      <c r="D1075" s="6"/>
+      <c r="E1075" s="5"/>
+      <c r="F1075" s="5"/>
+    </row>
+    <row r="1076" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1076" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1076" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1076" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1076" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1076" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1076" s="5"/>
+    </row>
+    <row r="1077" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1077" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1077" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1077" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1077" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1077" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1077" s="5"/>
+    </row>
+    <row r="1078" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1078" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1078" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1078" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1078" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1078" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1078" s="5"/>
+    </row>
+    <row r="1079" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1079" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1079" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1079" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1079" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1079" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1079" s="5"/>
+    </row>
+    <row r="1080" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1080" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1080" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C1080" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1080" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1080" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1080" s="11"/>
+    </row>
+    <row r="1081" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1081" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1081" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1081" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1081" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1081" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1081" s="11"/>
+    </row>
+    <row r="1082" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1082" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1082" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1082" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1082" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1082" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1082" s="5"/>
+    </row>
+    <row r="1083" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1083" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1083" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C1083" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1083" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1083" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1083" s="5"/>
+    </row>
+    <row r="1084" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1084" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="B1084" s="5"/>
+      <c r="C1084" s="5"/>
+      <c r="D1084" s="6"/>
+      <c r="E1084" s="5"/>
+      <c r="F1084" s="5"/>
+    </row>
+    <row r="1085" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1085" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1085" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1085" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1085" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1085" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1085" s="5"/>
+    </row>
+    <row r="1086" spans="1:6" ht="21" thickBot="1" x14ac:dyDescent="0.8">
+      <c r="A1086" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1086" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1086" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1086" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1086" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1086" s="12"/>
+    </row>
+    <row r="1087" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1087" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1087" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C1087" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1087" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1087" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1087" s="5"/>
+    </row>
+    <row r="1088" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1088" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1088" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1088" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1088" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1088" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1088" s="5"/>
+    </row>
+    <row r="1089" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1089" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1089" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1089" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1089" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1089" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1089" s="5"/>
+    </row>
+    <row r="1090" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1090" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1090" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1090" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1090" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1090" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1090" s="5"/>
+    </row>
+    <row r="1091" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1091" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1091" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1091" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1091" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1091" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1091" s="11"/>
+    </row>
+    <row r="1092" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1092" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1092" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1092" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1092" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1092" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1092" s="11"/>
+    </row>
+    <row r="1093" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1093" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="B1093" s="5"/>
+      <c r="C1093" s="5"/>
+      <c r="D1093" s="6"/>
+      <c r="E1093" s="5"/>
+      <c r="F1093" s="5"/>
+    </row>
+    <row r="1094" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1094" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1094" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1094" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1094" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1094" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1094" s="5"/>
+    </row>
+    <row r="1095" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1095" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1095" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="C1095" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1095" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1095" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1095" s="5"/>
+    </row>
+    <row r="1096" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1096" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1096" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="C1096" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1096" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1096" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1096" s="11"/>
+    </row>
+    <row r="1097" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1097" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1097" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C1097" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1097" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1097" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1097" s="11"/>
+    </row>
+    <row r="1098" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1098" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1098" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1098" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D1098" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1098" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1098" s="5"/>
+    </row>
+    <row r="1099" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1099" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1099" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="C1099" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1099" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1099" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1099" s="11"/>
+    </row>
+    <row r="1100" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1100" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1100" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1100" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1100" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1100" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1100" s="13"/>
+    </row>
+    <row r="1101" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1101" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1101" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1101" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1101" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1101" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1101" s="13"/>
+    </row>
+    <row r="1102" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1102" s="5" t="s">
+        <v>817</v>
+      </c>
+      <c r="B1102" s="5"/>
+      <c r="C1102" s="5"/>
+      <c r="D1102" s="6"/>
+      <c r="E1102" s="5"/>
+      <c r="F1102" s="5"/>
+    </row>
+    <row r="1103" spans="1:6" ht="21.4" x14ac:dyDescent="0.8">
+      <c r="A1103" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1103" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="C1103" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1103" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1103" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1103" s="14"/>
+    </row>
+    <row r="1104" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1104" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1104" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="C1104" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1104" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1104" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1104" s="5"/>
+    </row>
+    <row r="1105" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1105" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1105" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C1105" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1105" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1105" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="F1105" s="5"/>
+    </row>
+    <row r="1106" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1106" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1106" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C1106" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1106" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1106" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="F1106" s="5"/>
+    </row>
+    <row r="1107" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1107" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1107" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C1107" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1107" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1107" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="F1107" s="5"/>
+    </row>
+    <row r="1108" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1108" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1108" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1108" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1108" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1108" s="5" t="s">
+        <v>821</v>
+      </c>
+      <c r="F1108" s="5"/>
+    </row>
+    <row r="1109" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1109" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1109" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1109" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1109" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1109" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1109" s="11"/>
+    </row>
+    <row r="1110" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1110" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1110" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1110" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D1110" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1110" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1110" s="11"/>
+    </row>
+    <row r="1111" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1111" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="B1111" s="5"/>
+      <c r="C1111" s="5"/>
+      <c r="D1111" s="6"/>
+      <c r="E1111" s="5"/>
+      <c r="F1111" s="5"/>
+    </row>
+    <row r="1112" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1112" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1112" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1112" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1112" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1112" s="5" t="s">
+        <v>823</v>
+      </c>
+      <c r="F1112" s="11"/>
+    </row>
+    <row r="1113" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1113" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1113" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1113" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1113" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1113" s="5" t="s">
+        <v>824</v>
+      </c>
+      <c r="F1113" s="5"/>
+    </row>
+    <row r="1114" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1114" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1114" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1114" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D1114" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1114" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="F1114" s="11"/>
+    </row>
+    <row r="1115" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1115" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1115" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1115" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1115" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1115" s="5" t="s">
+        <v>826</v>
+      </c>
+      <c r="F1115" s="13"/>
+    </row>
+    <row r="1116" spans="1:6" ht="21.4" x14ac:dyDescent="0.8">
+      <c r="A1116" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1116" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1116" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="D1116" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1116" s="5" t="s">
+        <v>827</v>
+      </c>
+      <c r="F1116" s="14"/>
+    </row>
+    <row r="1117" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1117" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1117" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1117" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1117" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1117" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="F1117" s="11"/>
+    </row>
+    <row r="1118" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1118" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1118" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1118" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1118" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1118" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="F1118" s="5"/>
+    </row>
+    <row r="1119" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1119" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1119" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C1119" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1119" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1119" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="F1119" s="13"/>
+    </row>
+    <row r="1123" spans="1:6" ht="21.4" x14ac:dyDescent="0.8">
+      <c r="A1123" s="18"/>
+      <c r="B1123" s="19"/>
+      <c r="C1123" s="19"/>
+      <c r="D1123" s="20"/>
+      <c r="E1123" s="19"/>
+      <c r="F1123" s="21"/>
+    </row>
+    <row r="1124" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1124" s="22"/>
+      <c r="B1124" s="22"/>
+      <c r="C1124" s="22"/>
+      <c r="D1124" s="23"/>
+      <c r="E1124" s="22"/>
+      <c r="F1124" s="24"/>
+    </row>
+    <row r="1125" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1125" s="15"/>
+      <c r="B1125" s="15"/>
+      <c r="C1125" s="15"/>
+      <c r="D1125" s="16"/>
+      <c r="E1125" s="15"/>
+      <c r="F1125" s="17"/>
+    </row>
+    <row r="1126" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1126" s="15"/>
+      <c r="B1126" s="15"/>
+      <c r="C1126" s="15"/>
+      <c r="D1126" s="16"/>
+      <c r="E1126" s="15"/>
+      <c r="F1126" s="17"/>
+    </row>
+    <row r="1127" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1127" s="15"/>
+      <c r="B1127" s="15"/>
+      <c r="C1127" s="15"/>
+      <c r="D1127" s="16"/>
+      <c r="E1127" s="15"/>
+      <c r="F1127" s="17"/>
+    </row>
+    <row r="1128" spans="1:6" ht="20.65" x14ac:dyDescent="0.75">
+      <c r="A1128" s="15"/>
+      <c r="B1128" s="15"/>
+      <c r="C1128" s="15"/>
+      <c r="D1128" s="16"/>
+      <c r="E1128" s="15"/>
+      <c r="F1128" s="17"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>